<commit_message>
Update source data files with this afternoon's cleaned/refreshed exports
- DEPT_-_Master_Data(Sheet1).xlsx: 52 -> 50 rows
- UTILIZATION DATA SHEET.xlsx: 258 -> 1523 rows (extended date range)
- PowerBI_Ready_Utilization_May_2026.xlsx: restructured into named sheets
  (README, Employee_Weekly_Wide, Utilization_Long) instead of a single
  default sheet — matches the backend's already-updated data_loader.py /
  utilization_metrics.py, which reads GROUND_TRUTH_LONG_SHEET /
  GROUND_TRUTH_WIDE_SHEET by name. Utilization_Long is 164 rows, matching
  the documented ground-truth baseline.

Verified: all 148 backend tests pass against this data.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/data/PowerBI_Ready_Utilization_May_2026.xlsx
+++ b/backend/data/PowerBI_Ready_Utilization_May_2026.xlsx
@@ -758,12 +758,12 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n"/>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
+      <c r="A2" s="4" t="n"/>
+      <c r="B2" s="4" t="n"/>
+      <c r="C2" s="4" t="n"/>
+      <c r="D2" s="4" t="n"/>
+      <c r="E2" s="4" t="n"/>
+      <c r="F2" s="4" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -776,10 +776,10 @@
           <t>Purpose</t>
         </is>
       </c>
-      <c r="C3" s="2" t="n"/>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="n"/>
+      <c r="C3" s="4" t="n"/>
+      <c r="D3" s="4" t="n"/>
+      <c r="E3" s="4" t="n"/>
+      <c r="F3" s="4" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -792,10 +792,10 @@
           <t>One row per employee, with four weekly utilization columns plus the source period-total percentage.</t>
         </is>
       </c>
-      <c r="C4" s="2" t="n"/>
-      <c r="D4" s="2" t="n"/>
-      <c r="E4" s="2" t="n"/>
-      <c r="F4" s="2" t="n"/>
+      <c r="C4" s="4" t="n"/>
+      <c r="D4" s="4" t="n"/>
+      <c r="E4" s="4" t="n"/>
+      <c r="F4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -808,10 +808,10 @@
           <t>Recommended Power BI table: one row per employee per week.</t>
         </is>
       </c>
-      <c r="C5" s="2" t="n"/>
-      <c r="D5" s="2" t="n"/>
-      <c r="E5" s="2" t="n"/>
-      <c r="F5" s="2" t="n"/>
+      <c r="C5" s="4" t="n"/>
+      <c r="D5" s="4" t="n"/>
+      <c r="E5" s="4" t="n"/>
+      <c r="F5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -824,10 +824,10 @@
           <t>Department and grand-total rows from the source report were intentionally excluded because Power BI should calculate totals from employee rows.</t>
         </is>
       </c>
-      <c r="C6" s="2" t="n"/>
-      <c r="D6" s="2" t="n"/>
-      <c r="E6" s="2" t="n"/>
-      <c r="F6" s="2" t="n"/>
+      <c r="C6" s="4" t="n"/>
+      <c r="D6" s="4" t="n"/>
+      <c r="E6" s="4" t="n"/>
+      <c r="F6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -840,10 +840,10 @@
           <t>Blank weekly cells were preserved as blank; they were not converted to 0%.</t>
         </is>
       </c>
-      <c r="C7" s="2" t="n"/>
-      <c r="D7" s="2" t="n"/>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" s="2" t="n"/>
+      <c r="C7" s="4" t="n"/>
+      <c r="D7" s="4" t="n"/>
+      <c r="E7" s="4" t="n"/>
+      <c r="F7" s="4" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -856,10 +856,10 @@
           <t>The period-total percentage is retained from the source. It may be weighted and should not automatically be replaced with a simple average.</t>
         </is>
       </c>
-      <c r="C8" s="2" t="n"/>
-      <c r="D8" s="2" t="n"/>
-      <c r="E8" s="2" t="n"/>
-      <c r="F8" s="2" t="n"/>
+      <c r="C8" s="4" t="n"/>
+      <c r="D8" s="4" t="n"/>
+      <c r="E8" s="4" t="n"/>
+      <c r="F8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -872,10 +872,10 @@
           <t>Data was transcribed from screenshots, so please spot-check names and percentages against the original workbook before publishing.</t>
         </is>
       </c>
-      <c r="C9" s="2" t="n"/>
-      <c r="D9" s="2" t="n"/>
-      <c r="E9" s="2" t="n"/>
-      <c r="F9" s="2" t="n"/>
+      <c r="C9" s="4" t="n"/>
+      <c r="D9" s="4" t="n"/>
+      <c r="E9" s="4" t="n"/>
+      <c r="F9" s="4" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1540,7 +1540,7 @@
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>Kaginthala Reddy</t>
+          <t>Kagithala Reddy</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
@@ -2252,7 +2252,7 @@
       </c>
       <c r="C33" s="24" t="inlineStr">
         <is>
-          <t>Saumyarajan Kanungo</t>
+          <t>Saumyaranjan Kanungo</t>
         </is>
       </c>
       <c r="D33" s="24" t="inlineStr">
@@ -2336,7 +2336,7 @@
       </c>
       <c r="C35" s="24" t="inlineStr">
         <is>
-          <t>Suraj Kayade</t>
+          <t>Suraj Kavade</t>
         </is>
       </c>
       <c r="D35" s="24" t="inlineStr">
@@ -4878,7 +4878,7 @@
       </c>
       <c r="C62" s="11" t="inlineStr">
         <is>
-          <t>Kaginthala Reddy</t>
+          <t>Kagithala Reddy</t>
         </is>
       </c>
       <c r="D62" s="11" t="inlineStr">
@@ -4914,7 +4914,7 @@
       </c>
       <c r="C63" s="24" t="inlineStr">
         <is>
-          <t>Kaginthala Reddy</t>
+          <t>Kagithala Reddy</t>
         </is>
       </c>
       <c r="D63" s="24" t="inlineStr">
@@ -4950,7 +4950,7 @@
       </c>
       <c r="C64" s="11" t="inlineStr">
         <is>
-          <t>Kaginthala Reddy</t>
+          <t>Kagithala Reddy</t>
         </is>
       </c>
       <c r="D64" s="11" t="inlineStr">
@@ -4986,7 +4986,7 @@
       </c>
       <c r="C65" s="24" t="inlineStr">
         <is>
-          <t>Kaginthala Reddy</t>
+          <t>Kagithala Reddy</t>
         </is>
       </c>
       <c r="D65" s="24" t="inlineStr">
@@ -7470,7 +7470,7 @@
       </c>
       <c r="C134" s="11" t="inlineStr">
         <is>
-          <t>Saumyarajan Kanungo</t>
+          <t>Saumyaranjan Kanungo</t>
         </is>
       </c>
       <c r="D134" s="11" t="inlineStr">
@@ -7506,7 +7506,7 @@
       </c>
       <c r="C135" s="24" t="inlineStr">
         <is>
-          <t>Saumyarajan Kanungo</t>
+          <t>Saumyaranjan Kanungo</t>
         </is>
       </c>
       <c r="D135" s="24" t="inlineStr">
@@ -7542,7 +7542,7 @@
       </c>
       <c r="C136" s="11" t="inlineStr">
         <is>
-          <t>Saumyarajan Kanungo</t>
+          <t>Saumyaranjan Kanungo</t>
         </is>
       </c>
       <c r="D136" s="11" t="inlineStr">
@@ -7578,7 +7578,7 @@
       </c>
       <c r="C137" s="24" t="inlineStr">
         <is>
-          <t>Saumyarajan Kanungo</t>
+          <t>Saumyaranjan Kanungo</t>
         </is>
       </c>
       <c r="D137" s="24" t="inlineStr">
@@ -8190,7 +8190,7 @@
       </c>
       <c r="C154" s="11" t="inlineStr">
         <is>
-          <t>Suraj Kayade</t>
+          <t>Suraj Kavade</t>
         </is>
       </c>
       <c r="D154" s="11" t="inlineStr">
@@ -8226,7 +8226,7 @@
       </c>
       <c r="C155" s="24" t="inlineStr">
         <is>
-          <t>Suraj Kayade</t>
+          <t>Suraj Kavade</t>
         </is>
       </c>
       <c r="D155" s="24" t="inlineStr">
@@ -8262,7 +8262,7 @@
       </c>
       <c r="C156" s="11" t="inlineStr">
         <is>
-          <t>Suraj Kayade</t>
+          <t>Suraj Kavade</t>
         </is>
       </c>
       <c r="D156" s="11" t="inlineStr">
@@ -8298,7 +8298,7 @@
       </c>
       <c r="C157" s="24" t="inlineStr">
         <is>
-          <t>Suraj Kayade</t>
+          <t>Suraj Kavade</t>
         </is>
       </c>
       <c r="D157" s="24" t="inlineStr">

</xml_diff>

<commit_message>
Fix 'Pramod Kabugande' typo at source in ground-truth workbook
Corrected 5 cells (Utilization_Long + Employee_Weekly_Wide) to the
correct 'Pramod Kabugade' spelling that roster and booking already use,
and removed the now-stale BOOKING_TO_GROUND_TRUTH_NAME_MAP bridge that
only existed to paper over this typo during reconciliation (keeping it
would map booking's correct spelling to a name no longer in the ground
truth and drop those weeks). Surfaced by the Phase-8 cross-dataset
validation warning. Pre-fix workbook backed up under data/backups/.
Full suite 188 passed.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/data/PowerBI_Ready_Utilization_May_2026.xlsx
+++ b/backend/data/PowerBI_Ready_Utilization_May_2026.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employee_Weekly_Wide" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Utilization_Long" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Employee_Weekly_Wide" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Utilization_Long" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2588,7 +2588,7 @@
       </c>
       <c r="C41" s="24" t="inlineStr">
         <is>
-          <t>Pramod Kabugande</t>
+          <t>Pramod Kabugade</t>
         </is>
       </c>
       <c r="D41" s="24" t="inlineStr">
@@ -6174,7 +6174,7 @@
       </c>
       <c r="C98" s="11" t="inlineStr">
         <is>
-          <t>Pramod Kabugande</t>
+          <t>Pramod Kabugade</t>
         </is>
       </c>
       <c r="D98" s="11" t="inlineStr">
@@ -6210,7 +6210,7 @@
       </c>
       <c r="C99" s="24" t="inlineStr">
         <is>
-          <t>Pramod Kabugande</t>
+          <t>Pramod Kabugade</t>
         </is>
       </c>
       <c r="D99" s="24" t="inlineStr">
@@ -6246,7 +6246,7 @@
       </c>
       <c r="C100" s="11" t="inlineStr">
         <is>
-          <t>Pramod Kabugande</t>
+          <t>Pramod Kabugade</t>
         </is>
       </c>
       <c r="D100" s="11" t="inlineStr">
@@ -6282,7 +6282,7 @@
       </c>
       <c r="C101" s="24" t="inlineStr">
         <is>
-          <t>Pramod Kabugande</t>
+          <t>Pramod Kabugade</t>
         </is>
       </c>
       <c r="D101" s="24" t="inlineStr">

</xml_diff>